<commit_message>
better Turnierraster Style and PROTOKOLL.txt update
</commit_message>
<xml_diff>
--- a/additional Files/Piberdaten-test.xlsx
+++ b/additional Files/Piberdaten-test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\pro\GitHub\GitHub\ePiber\additional Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0B8F2DA-945B-437F-B3FE-41A00531BF4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E060036A-96F8-4309-B106-BFCC0B425F98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4965" yWindow="2700" windowWidth="21600" windowHeight="12645" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Personen" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1220" uniqueCount="897">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1225" uniqueCount="902">
   <si>
     <t>ID</t>
   </si>
@@ -2719,13 +2719,28 @@
   </si>
   <si>
     <t>260616-0808</t>
+  </si>
+  <si>
+    <t>260624-1515</t>
+  </si>
+  <si>
+    <t>260622-1045</t>
+  </si>
+  <si>
+    <t>R2-P1</t>
+  </si>
+  <si>
+    <t>6-3/6-1</t>
+  </si>
+  <si>
+    <t>6-3/6-2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -2749,6 +2764,12 @@
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2786,7 +2807,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2796,6 +2817,7 @@
     <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -10597,10 +10619,10 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:M999"/>
+  <dimension ref="A1:N999"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -10640,8 +10662,11 @@
       <c r="M1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="N1" s="5" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -10670,7 +10695,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:13" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -10699,7 +10724,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:13" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -10728,7 +10753,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -10751,7 +10776,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -10774,7 +10799,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -10797,7 +10822,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -10820,7 +10845,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -10843,7 +10868,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -10866,7 +10891,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -10889,7 +10914,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -10912,7 +10937,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -10935,7 +10960,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -10958,7 +10983,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -10981,7 +11006,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -11004,7 +11029,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -11027,7 +11052,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -11050,7 +11075,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -11073,7 +11098,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -11096,7 +11121,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
@@ -11119,7 +11144,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
@@ -11142,7 +11167,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
@@ -11165,7 +11190,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
@@ -11188,7 +11213,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
@@ -11211,7 +11236,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -11234,7 +11259,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>23</v>
       </c>
@@ -11257,11 +11282,67 @@
         <v>137</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="12.75" x14ac:dyDescent="0.2"/>
-    <row r="29" spans="1:13" ht="12.75" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:13" ht="12.75" x14ac:dyDescent="0.2"/>
-    <row r="31" spans="1:13" ht="12.75" x14ac:dyDescent="0.2"/>
-    <row r="32" spans="1:13" ht="12.75" x14ac:dyDescent="0.2"/>
+    <row r="28" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>33</v>
+      </c>
+      <c r="B28" t="s">
+        <v>763</v>
+      </c>
+      <c r="C28" t="s">
+        <v>764</v>
+      </c>
+      <c r="D28">
+        <v>5</v>
+      </c>
+      <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="H28">
+        <v>42</v>
+      </c>
+      <c r="J28" t="s">
+        <v>900</v>
+      </c>
+      <c r="M28">
+        <v>42</v>
+      </c>
+      <c r="N28" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>34</v>
+      </c>
+      <c r="B29" t="s">
+        <v>766</v>
+      </c>
+      <c r="C29" t="s">
+        <v>767</v>
+      </c>
+      <c r="D29">
+        <v>5</v>
+      </c>
+      <c r="F29">
+        <v>2</v>
+      </c>
+      <c r="H29">
+        <v>41</v>
+      </c>
+      <c r="J29" t="s">
+        <v>901</v>
+      </c>
+      <c r="M29">
+        <v>2</v>
+      </c>
+      <c r="N29" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="12.75" x14ac:dyDescent="0.2"/>
+    <row r="31" spans="1:14" ht="12.75" x14ac:dyDescent="0.2"/>
+    <row r="32" spans="1:14" ht="12.75" x14ac:dyDescent="0.2"/>
     <row r="33" ht="12.75" x14ac:dyDescent="0.2"/>
     <row r="34" ht="12.75" x14ac:dyDescent="0.2"/>
     <row r="35" ht="12.75" x14ac:dyDescent="0.2"/>
@@ -12506,420 +12587,395 @@
     </row>
     <row r="12" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A12">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B12" t="s">
-        <v>763</v>
+        <v>769</v>
       </c>
       <c r="C12" t="s">
-        <v>764</v>
+        <v>770</v>
       </c>
       <c r="D12">
         <v>5</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H12">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="J12" t="s">
         <v>36</v>
       </c>
       <c r="K12" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A13">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B13" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
       <c r="C13" t="s">
-        <v>767</v>
+        <v>773</v>
       </c>
       <c r="D13">
         <v>5</v>
       </c>
       <c r="F13">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H13">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="J13" t="s">
         <v>36</v>
       </c>
       <c r="K13" t="s">
-        <v>768</v>
+        <v>774</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A14">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B14" t="s">
-        <v>769</v>
+        <v>775</v>
       </c>
       <c r="C14" t="s">
-        <v>770</v>
+        <v>776</v>
       </c>
       <c r="D14">
         <v>5</v>
       </c>
       <c r="F14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H14">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="J14" t="s">
         <v>36</v>
       </c>
       <c r="K14" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A15">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B15" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
       <c r="C15" t="s">
-        <v>773</v>
+        <v>779</v>
       </c>
       <c r="D15">
         <v>5</v>
       </c>
       <c r="F15">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H15">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="J15" t="s">
         <v>36</v>
       </c>
       <c r="K15" t="s">
-        <v>774</v>
+        <v>780</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A16">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>775</v>
+        <v>781</v>
       </c>
       <c r="C16" t="s">
-        <v>776</v>
+        <v>782</v>
       </c>
       <c r="D16">
         <v>5</v>
       </c>
       <c r="F16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H16">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="J16" t="s">
         <v>36</v>
       </c>
       <c r="K16" t="s">
-        <v>777</v>
+        <v>783</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A17">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="B17" t="s">
-        <v>778</v>
+        <v>784</v>
       </c>
       <c r="C17" t="s">
-        <v>779</v>
+        <v>785</v>
       </c>
       <c r="D17">
         <v>5</v>
       </c>
       <c r="F17">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H17">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="J17" t="s">
         <v>36</v>
       </c>
       <c r="K17" t="s">
-        <v>780</v>
+        <v>786</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A18">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="B18" t="s">
-        <v>781</v>
+        <v>787</v>
       </c>
       <c r="C18" t="s">
-        <v>782</v>
+        <v>788</v>
       </c>
       <c r="D18">
         <v>5</v>
       </c>
       <c r="F18">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H18">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J18" t="s">
         <v>36</v>
       </c>
       <c r="K18" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A19">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="B19" t="s">
-        <v>784</v>
+        <v>790</v>
       </c>
       <c r="C19" t="s">
-        <v>785</v>
+        <v>791</v>
       </c>
       <c r="D19">
         <v>5</v>
       </c>
       <c r="F19">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H19">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="J19" t="s">
         <v>36</v>
       </c>
       <c r="K19" t="s">
-        <v>786</v>
+        <v>792</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A20">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="B20" t="s">
-        <v>787</v>
+        <v>793</v>
       </c>
       <c r="C20" t="s">
-        <v>788</v>
+        <v>794</v>
       </c>
       <c r="D20">
         <v>5</v>
       </c>
       <c r="F20">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H20">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J20" t="s">
         <v>36</v>
       </c>
       <c r="K20" t="s">
-        <v>789</v>
+        <v>795</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A21">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="B21" t="s">
-        <v>790</v>
+        <v>796</v>
       </c>
       <c r="C21" t="s">
-        <v>791</v>
+        <v>797</v>
       </c>
       <c r="D21">
         <v>5</v>
       </c>
       <c r="F21">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H21">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J21" t="s">
         <v>36</v>
       </c>
       <c r="K21" t="s">
-        <v>792</v>
+        <v>798</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A22">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="B22" t="s">
-        <v>793</v>
+        <v>799</v>
       </c>
       <c r="C22" t="s">
-        <v>794</v>
+        <v>800</v>
       </c>
       <c r="D22">
         <v>5</v>
       </c>
       <c r="F22">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H22">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J22" t="s">
         <v>36</v>
       </c>
       <c r="K22" t="s">
-        <v>795</v>
+        <v>801</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A23">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="B23" t="s">
-        <v>796</v>
+        <v>802</v>
       </c>
       <c r="C23" t="s">
-        <v>797</v>
+        <v>803</v>
       </c>
       <c r="D23">
         <v>5</v>
       </c>
       <c r="F23">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H23">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="J23" t="s">
         <v>36</v>
       </c>
       <c r="K23" t="s">
-        <v>798</v>
+        <v>804</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A24">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="B24" t="s">
-        <v>799</v>
+        <v>805</v>
       </c>
       <c r="C24" t="s">
-        <v>800</v>
+        <v>806</v>
       </c>
       <c r="D24">
         <v>5</v>
       </c>
       <c r="F24">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H24">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="J24" t="s">
         <v>36</v>
       </c>
       <c r="K24" t="s">
-        <v>801</v>
+        <v>807</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A25">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="B25" t="s">
-        <v>802</v>
+        <v>808</v>
       </c>
       <c r="C25" t="s">
-        <v>803</v>
+        <v>809</v>
       </c>
       <c r="D25">
         <v>5</v>
       </c>
       <c r="F25">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H25">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J25" t="s">
         <v>36</v>
       </c>
       <c r="K25" t="s">
-        <v>804</v>
+        <v>810</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A26">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="B26" t="s">
-        <v>805</v>
+        <v>897</v>
       </c>
       <c r="C26" t="s">
-        <v>806</v>
+        <v>898</v>
       </c>
       <c r="D26">
         <v>5</v>
       </c>
       <c r="F26">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="H26">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="J26" t="s">
         <v>36</v>
       </c>
       <c r="K26" t="s">
-        <v>807</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A27">
-        <v>33</v>
-      </c>
-      <c r="B27" t="s">
-        <v>808</v>
-      </c>
-      <c r="C27" t="s">
-        <v>809</v>
-      </c>
-      <c r="D27">
-        <v>5</v>
-      </c>
-      <c r="F27">
-        <v>16</v>
-      </c>
-      <c r="H27">
-        <v>27</v>
-      </c>
-      <c r="J27" t="s">
-        <v>36</v>
-      </c>
-      <c r="K27" t="s">
-        <v>810</v>
-      </c>
-    </row>
+        <v>899</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="12.75" x14ac:dyDescent="0.2"/>
     <row r="28" spans="1:11" ht="12.75" x14ac:dyDescent="0.2"/>
     <row r="29" spans="1:11" ht="12.75" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:11" ht="12.75" x14ac:dyDescent="0.2"/>

</xml_diff>